<commit_message>
Update port configuration workbook with latest UO and zone data.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data_modelos/1_Configuración_del_puerto.xlsx
+++ b/data_modelos/1_Configuración_del_puerto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PDE\DEMO\data_modelos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2FBEB2F-571C-4DD3-8FA9-32385A9F312C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E3F55F5-58AA-4ACD-ACF9-12ECE96E86DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$9:$D$13</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$A$1:$I$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$A$1:$I$29</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -128,7 +128,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="39">
   <si>
     <t>Zona de fondeo y espera exterior</t>
   </si>
@@ -294,7 +294,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -315,17 +315,6 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -359,9 +348,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -650,7 +637,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -743,7 +730,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
-        <f t="shared" ref="A4:A28" si="0">+A3+1</f>
+        <f t="shared" ref="A4:A29" si="0">+A3+1</f>
         <v>3</v>
       </c>
       <c r="B4" s="2">
@@ -1375,7 +1362,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>5</v>
@@ -1386,13 +1373,40 @@
       <c r="E28" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="F28" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G28" t="s">
-        <v>16</v>
-      </c>
-      <c r="H28" t="s">
+      <c r="F28" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G28" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H28" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="B29" s="2">
+        <v>1</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H29" s="10" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1403,7 +1417,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E28" xr:uid="{0F46184E-0E40-4450-9C61-1B1892F4990F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E29" xr:uid="{0F46184E-0E40-4450-9C61-1B1892F4990F}">
       <formula1>"Activo físico, Operacional (servicios)"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>